<commit_message>
Anpassung auf neue Datenbasis von 24 bis 26
</commit_message>
<xml_diff>
--- a/data/processed/mta_mapping_bemerkung.xlsx
+++ b/data/processed/mta_mapping_bemerkung.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C184"/>
+  <dimension ref="A1:C219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,102 +436,102 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>515102786 stirnwände (niedrige höhe)op120.1 schweißung querträger oben r06/r07 achsen sollgeschwindigkeit überschritten</t>
+          <t>1 schweißer</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>515102786 stirnwände (niedrige höhe)op120.1 schweißung querträger oben r06/r07 achsen sollgeschwindigkeit überschritten</t>
+          <t>1 schweißer</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>anlage auffüllen</t>
+          <t>515102786 stirnwände (niedrige höhe)op120.1 schweißung querträger oben r06/r07 achsen sollgeschwindigkeit überschritten</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>anlage auffüllen</t>
+          <t>515102786 stirnwände (niedrige höhe)op120.1 schweißung querträger oben r06/r07 achsen sollgeschwindigkeit überschritten</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>anlage leer (keine eckrungen mehr vorhanden)</t>
+          <t>anlage auffüllen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>anlage leer (keine eckrungen mehr vorhanden)</t>
+          <t>anlage auffüllen</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>anlage leer gelaufen auffüllen</t>
+          <t>anlage leer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>anlage leer gelaufen auffüllen</t>
+          <t>anlage leer</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>anlage voll gefahren</t>
+          <t>anlage leer (keine eckrungen mehr vorhanden)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>anlage voll gefahren</t>
+          <t>anlage leer (keine eckrungen mehr vorhanden)</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>anlage wieder vollfahren</t>
+          <t>anlage leer gelaufen auffüllen</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>anlage wieder vollfahren</t>
+          <t>anlage leer gelaufen auffüllen</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>anlagenreinigung</t>
+          <t>anlage mit störung übernommen</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>anlagenreinigung</t>
+          <t>anlage mit störung übernommen</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -541,42 +541,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>anlagenreinigung/robtechs in der anlage</t>
+          <t>anlage voll fahren</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>anlagenreinigung/robtechs in der anlage</t>
+          <t>anlage voll fahren</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>aufträge mit 5 knoten - position nacharbeiten</t>
+          <t>anlage voll gefahren</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>aufträge mit 5 knoten - position nacharbeiten</t>
+          <t>anlage voll gefahren</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>aushubsstörung nachdem der schlitten komplett runtergefallen ist, robotertechniker informiert, kabel defekt</t>
+          <t>anlage wieder auffüllen</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>aushubsstörung nachdem der schlitten komplett runtergefallen ist, robotertechniker informiert, kabel defekt</t>
+          <t>anlage wieder auffüllen</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -586,27 +586,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>bauteil nicht gespannt</t>
+          <t>anlage wieder vollfahren</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bauteil nicht gespannt</t>
+          <t>anlage wieder vollfahren</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>bauteil wird nicht gespannt, stütze schiebt sich über den anschlag</t>
+          <t>anlagenbereich fegen</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>bauteil wird nicht gespannt, stütze schiebt sich über den anschlag</t>
+          <t>anlagenbereich fegen</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -616,12 +616,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>bauteil wird nicht gespannt-instandsetzung informiert</t>
+          <t>anlagenreinigung</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bauteil wird nicht gespannt-instandsetzung informiert</t>
+          <t>anlagenreinigung</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -631,57 +631,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>bauteilspanner spannen nicht</t>
+          <t>anlagenreinigung/robtechs in der anlage</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>bauteilspanner spannen nicht</t>
+          <t>anlagenreinigung/robtechs in der anlage</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>bedienerschutz ausgelöst</t>
+          <t>aufträge mit 5 knoten - position nacharbeiten</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>bedienerschutz ausgelöst</t>
+          <t>aufträge mit 5 knoten - position nacharbeiten</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>bedienerschutz ausgelöst folgefehler beseitigen</t>
+          <t>aushubsstörung nachdem der schlitten komplett runtergefallen ist, robotertechniker informiert, kabel defekt</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>bedienerschutz ausgelöst folgefehler beseitigen</t>
+          <t>aushubsstörung nachdem der schlitten komplett runtergefallen ist, robotertechniker informiert, kabel defekt</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>bedienerschutz-folgefehler beseitigen</t>
+          <t>bauteil nicht gespannt</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>bedienerschutz-folgefehler beseitigen</t>
+          <t>bauteil nicht gespannt</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -691,57 +691,57 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>beim tb kommissionieren, sensoren links ab und anklemmen</t>
+          <t>bauteil wird nicht gespannt, stütze schiebt sich über den anschlag</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>beim tb kommissionieren, sensoren links ab und anklemmen</t>
+          <t>bauteil wird nicht gespannt, stütze schiebt sich über den anschlag</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bekommt kein signal von op 120 (systemabsturz)</t>
+          <t>bauteil wird nicht gespannt-instandsetzung informiert</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>bekommt kein signal von op 120 (systemabsturz)</t>
+          <t>bauteil wird nicht gespannt-instandsetzung informiert</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>bekommt keinen auftrag</t>
+          <t>bauteilspanner spannen nicht</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>bekommt keinen auftrag</t>
+          <t>bauteilspanner spannen nicht</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>bleche anmelden und sensoren ab und an schrauben</t>
+          <t>bedienerschutz ausgelöst</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>bleche anmelden und sensoren ab und an schrauben</t>
+          <t>bedienerschutz ausgelöst</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -751,27 +751,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>bleche beladen</t>
+          <t>bedienerschutz ausgelöst folgefehler beseitigen</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>bleche beladen</t>
+          <t>bedienerschutz ausgelöst folgefehler beseitigen</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>bleche einlagern</t>
+          <t>bedienerschutz-folgefehler beseitigen.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>bleche einlagern</t>
+          <t>bedienerschutz-folgefehler beseitigen.</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -781,57 +781,57 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>bleche nicht richtig gespannt</t>
+          <t>beim tb kommissionieren, sensoren links ab und anklemmen .</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>bleche nicht richtig gespannt</t>
+          <t>beim tb kommissionieren, sensoren links ab und anklemmen .</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>bleche räumen =&gt; anlage leergelaufen</t>
+          <t>bekommt kein signal von op 120 (systemabsturz)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>bleche räumen =&gt; anlage leergelaufen</t>
+          <t>bekommt kein signal von op 120 (systemabsturz)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>bmb führt optimierungsarbeiten</t>
+          <t>bekommt keinen auftrag</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>bmb führt optimierungsarbeiten</t>
+          <t>bekommt keinen auftrag</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>bmb und fa. fronius bei der anlage</t>
+          <t>bleche anmelden und sensoren ab und an schrauben</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>bmb und fa. fronius bei der anlage</t>
+          <t>bleche anmelden und sensoren ab und an schrauben</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -841,57 +841,57 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>brennerkollision</t>
+          <t>bleche beladen</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>brennerkollision</t>
+          <t>bleche beladen</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>collision detected</t>
+          <t>bleche einlagern</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>collision detected</t>
+          <t>bleche einlagern</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>drahtfass wechseln</t>
+          <t>bleche kleben aneinander</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>drahtfass wechseln</t>
+          <t>bleche kleben aneinander</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>drahtfasswechsel/sele reinigen</t>
+          <t>bleche manuell laden</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>drahtfasswechsel/sele reinigen</t>
+          <t>bleche manuell laden</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -901,27 +901,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>drahtfestbrand</t>
+          <t>bleche nicht richtig gespannt</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>drahtfestbrand</t>
+          <t>bleche nicht richtig gespannt</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>drahtfestbrand (strom und gasdüse getauscht)</t>
+          <t>bleche räumen =&gt; anlage leergelaufen</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>drahtfestbrand (strom und gasdüse getauscht)</t>
+          <t>bleche räumen =&gt; anlage leergelaufen</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -931,27 +931,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>drahtfestbrand op120-2 (stromdüse getauscht)</t>
+          <t>bmb führt optimierungsarbeiten</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>drahtfestbrand op120-2 (stromdüse getauscht)</t>
+          <t>bmb führt optimierungsarbeiten</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>drahtfestbrand op120.1 (stromdüse gereinigt)</t>
+          <t>bmb und fa. fronius bei der anlage</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>drahtfestbrand op120.1 (stromdüse gereinigt)</t>
+          <t>bmb und fa. fronius bei der anlage</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -961,117 +961,117 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>drahttone wechseln =&gt; keine ameise</t>
+          <t>brennerkollision</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>drahttone wechseln =&gt; keine ameise</t>
+          <t>brennerkollision</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>fehler schrittkette</t>
+          <t>collision detected</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>fehler schrittkette</t>
+          <t>collision detected</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>fronius störung/stromdüse festgebrannt</t>
+          <t>drahtfass wechseln</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>fronius störung/stromdüse festgebrannt</t>
+          <t>drahtfass wechseln</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>fährt kollisionen softwareendschalter a3</t>
+          <t>drahtfasswechsel/sele reinigen</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>fährt kollisionen softwareendschalter a3</t>
+          <t>drahtfasswechsel/sele reinigen</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>fährt kollisionen softwareendschalter a3 (robotertechniker hat positionen angepasst/ große stw r6 zu nah vorm skid)</t>
+          <t>drahtfestbrand</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>fährt kollisionen softwareendschalter a3 (robotertechniker hat positionen angepasst/ große stw r6 zu nah vorm skid)</t>
+          <t>drahtfestbrand</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>gestell mit 229 in der anlage hatte 1 blech zu wenig eingelagert, das folge gestell mit 229 makiert hatte die bleche falsch eingebucht statt 229 waren es 230 ( durch frühschicht )</t>
+          <t>drahtfestbrand (strom und gasdüse getauscht)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>gestell mit 229 in der anlage hatte 1 blech zu wenig eingelagert, das folge gestell mit 229 makiert hatte die bleche falsch eingebucht statt 229 waren es 230 ( durch frühschicht )</t>
+          <t>drahtfestbrand (strom und gasdüse getauscht)</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>greifer fährt in leere palette (logistik falsch gezählt)</t>
+          <t>drahtfestbrand op120-2 (stromdüse getauscht)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>greifer fährt in leere palette (logistik falsch gezählt)</t>
+          <t>drahtfestbrand op120-2 (stromdüse getauscht)</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>greifer wegen vakuumstörungen instandsetzen</t>
+          <t>drahtfestbrand op120.1 (stromdüse gereinigt)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>greifer wegen vakuumstörungen instandsetzen</t>
+          <t>drahtfestbrand op120.1 (stromdüse gereinigt)</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1081,12 +1081,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>info-ansprache</t>
+          <t>drahttone wechseln =&gt; keine ameise</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>info-ansprache</t>
+          <t>drahttone wechseln =&gt; keine ameise</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1096,12 +1096,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>kabelbruch/störung in der steuerung instandsetzung informiert-warten auf techniker</t>
+          <t>es wurde versucht das zuständige personal telefonisch zu erreichen, ohne erfolg</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>kabelbruch/störung in der steuerung instandsetzung informiert-warten auf techniker</t>
+          <t>es wurde versucht das zuständige personal telefonisch zu erreichen, ohne erfolg</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1111,12 +1111,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>kein vakuum</t>
+          <t>falsche bleche in der anlage</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>kein vakuum</t>
+          <t>falsche bleche in der anlage</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1126,12 +1126,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>kein vakuum - bleche zu ölig</t>
+          <t>fehler schrittkette</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>kein vakuum - bleche zu ölig</t>
+          <t>fehler schrittkette</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1141,72 +1141,72 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>keine gestelle</t>
+          <t>festgebrannt</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>keine gestelle</t>
+          <t>festgebrannt</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>keine qt. oben l5 515136662 (anlage leer)</t>
+          <t>fronius störung/stromdüse festgebrannt</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>keine qt. oben l5 515136662 (anlage leer)</t>
+          <t>fronius störung/stromdüse festgebrannt</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>keine rungen/keine trapezbleche/</t>
+          <t>fährt kollisionen softwareendschalter a3</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>keine rungen/keine trapezbleche/</t>
+          <t>fährt kollisionen softwareendschalter a3</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>keine stützfüße liner 5 mehr vorhanden, produzieren auf palette ohne er</t>
+          <t>fährt kollisionen softwareendschalter a3 (robotertechniker hat positionen angepasst/ große stw r6 zu nah vorm skid)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>keine stützfüße liner 5 mehr vorhanden, produzieren auf palette ohne er</t>
+          <t>fährt kollisionen softwareendschalter a3 (robotertechniker hat positionen angepasst/ große stw r6 zu nah vorm skid)</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>klammer-schlitten unten nicht gelöst</t>
+          <t>gestell mit 229 in der anlage hatte 1 blech zu wenig eingelagert, das folge gestell mit 229 makiert hatte die bleche falsch eingebucht statt 229 waren es 230 ( durch frühschicht )</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>klammer-schlitten unten nicht gelöst</t>
+          <t>gestell mit 229 in der anlage hatte 1 blech zu wenig eingelagert, das folge gestell mit 229 makiert hatte die bleche falsch eingebucht statt 229 waren es 230 ( durch frühschicht )</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -1216,12 +1216,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>knoten im drahtfass, draht kann nicht gefördert werden</t>
+          <t>greifer fährt in leere palette (logistik falsch gezählt)</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>knoten im drahtfass, draht kann nicht gefördert werden</t>
+          <t>greifer fährt in leere palette (logistik falsch gezählt)</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -1231,27 +1231,27 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>knotengreifer 1 instandsetzen</t>
+          <t>greifer wegen vakuumstörungen instandsetzen</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>knotengreifer 1 instandsetzen</t>
+          <t>greifer wegen vakuumstörungen instandsetzen</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>knotengreifer 1 sensor schaltet nicht</t>
+          <t>info-ansprache</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>knotengreifer 1 sensor schaltet nicht</t>
+          <t>info-ansprache</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1261,12 +1261,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>knotengreifer 1 störung, robotertechniker informiert</t>
+          <t>instandsetzung führt reperaturen durch</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>knotengreifer 1 störung, robotertechniker informiert</t>
+          <t>instandsetzung führt reperaturen durch</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1276,12 +1276,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>knotengreifer störung in op70 sowie op50, robotertechniker informiert und einstellen lassen</t>
+          <t>intsandsetzung in der anlage</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>knotengreifer störung in op70 sowie op50, robotertechniker informiert und einstellen lassen</t>
+          <t>intsandsetzung in der anlage</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -1291,117 +1291,117 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>kolision</t>
+          <t>kabelbruch/störung in der steuerung instandsetzung informiert-warten auf techniker</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>kolision</t>
+          <t>kabelbruch/störung in der steuerung instandsetzung informiert-warten auf techniker</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>kollision</t>
+          <t>kein bediener</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>kollision</t>
+          <t>kein bediener</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>kollision / brenner tauschen</t>
+          <t>kein vakuum</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>kollision / brenner tauschen</t>
+          <t>kein vakuum</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>kollision bei 5 knoten schweißen</t>
+          <t>kein vakuum - bleche zu ölig</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>kollision bei 5 knoten schweißen</t>
+          <t>kein vakuum - bleche zu ölig</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>kollision detected</t>
+          <t>kein vakuum op130.2</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>kollision detected</t>
+          <t>kein vakuum op130.2</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>kollision op120.1/r06 kollision/r05 vakuum</t>
+          <t>keine gestelle</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>kollision op120.1/r06 kollision/r05 vakuum</t>
+          <t>keine gestelle</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>kollision op130-1</t>
+          <t>keine qt. oben l5 515136662 (anlage leer)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>kollision op130-1</t>
+          <t>keine qt. oben l5 515136662 (anlage leer)</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>kollisionsabfrage in op 120.1</t>
+          <t>keine rungen/keine trapezbleche/</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>kollisionsabfrage in op 120.1</t>
+          <t>keine rungen/keine trapezbleche/</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -1411,117 +1411,117 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>kran störung, fernbedienung funktioniert nicht mehr elektriker informiert</t>
+          <t>keine stützfüße liner 5 mehr vorhanden, produzieren auf palette ohne er.</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>kran störung, fernbedienung funktioniert nicht mehr elektriker informiert</t>
+          <t>keine stützfüße liner 5 mehr vorhanden, produzieren auf palette ohne er.</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>leoni</t>
+          <t>klammer-schlitten unten nicht gelöst</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>leoni</t>
+          <t>klammer-schlitten unten nicht gelöst</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>leoni störung</t>
+          <t>knoten im drahtfass, draht kann nicht gefördert werden</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>leoni störung</t>
+          <t>knoten im drahtfass, draht kann nicht gefördert werden</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>leoni-fehler</t>
+          <t>knotengreifer 1 instandsetzen</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>leoni-fehler</t>
+          <t>knotengreifer 1 instandsetzen</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>lichtbogen konnte nicht erzeugt werden</t>
+          <t>knotengreifer 1 sensor schaltet nicht</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>lichtbogen konnte nicht erzeugt werden</t>
+          <t>knotengreifer 1 sensor schaltet nicht</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>mehrere stw 5 knoten op50 ist langsamer &amp; ( 5.ten knoten umsetzen)</t>
+          <t>knotengreifer 1 störung, robotertechniker informiert</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>mehrere stw 5 knoten op50 ist langsamer &amp; ( 5.ten knoten umsetzen)</t>
+          <t>knotengreifer 1 störung, robotertechniker informiert</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>mes - absturz keine etiketten-manuel ausdruken</t>
+          <t>knotengreifer störung in op70 sowie op50, robotertechniker informiert und einstellen lassen</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>mes - absturz keine etiketten-manuel ausdruken</t>
+          <t>knotengreifer störung in op70 sowie op50, robotertechniker informiert und einstellen lassen</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>mitarbeitergespräch mit früh und spätschicht</t>
+          <t>kolision</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>mitarbeitergespräch mit früh und spätschicht</t>
+          <t>kolision</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -1531,27 +1531,27 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>mittelnaht mangelhaft</t>
+          <t>kollision</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>mittelnaht mangelhaft</t>
+          <t>kollision</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>mittelnaht schlecht robotertechniker informiert</t>
+          <t>kollision / brenner tauschen</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>mittelnaht schlecht robotertechniker informiert</t>
+          <t>kollision / brenner tauschen</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -1561,87 +1561,87 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>not-aus</t>
+          <t>kollision bei 5 knoten schweißen</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>not-aus</t>
+          <t>kollision bei 5 knoten schweißen</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>not-aus folgefehler beseitigen</t>
+          <t>kollision detected</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>not-aus folgefehler beseitigen</t>
+          <t>kollision detected</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>not-aus-durch monteur op100 folgefehler beseitigen</t>
+          <t>kollision op120.1/r06 kollision/r05 vakuum</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>not-aus-durch monteur op100 folgefehler beseitigen</t>
+          <t>kollision op120.1/r06 kollision/r05 vakuum</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>obenquerträger+trapezblech 5mm spalt=&gt; schweißnähte mangelhaft</t>
+          <t>kollision op130-1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>obenquerträger+trapezblech 5mm spalt=&gt; schweißnähte mangelhaft</t>
+          <t>kollision op130-1</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>op10. r. kein vakuum-bleche manuell laden</t>
+          <t>kollisionsabfrage in op 120.1</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>op10. r. kein vakuum-bleche manuell laden</t>
+          <t>kollisionsabfrage in op 120.1</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>op120.1 auf passiv gestellt, reparaturarbeiten</t>
+          <t>kran störung, fernbedienung funktioniert nicht mehr elektriker informiert</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>op120.1 auf passiv gestellt, reparaturarbeiten</t>
+          <t>kran störung, fernbedienung funktioniert nicht mehr elektriker informiert</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -1651,12 +1651,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>op130.2 auf passiv gestellt, reparaturarbeiten ( zylinder tauschen)</t>
+          <t>leertakt beim wechsel von liner 4 zu liner 5</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>op130.2 auf passiv gestellt, reparaturarbeiten ( zylinder tauschen)</t>
+          <t>leertakt beim wechsel von liner 4 zu liner 5</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -1666,57 +1666,57 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>optimierungsarbeiten an der anlage</t>
+          <t>leoni</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>optimierungsarbeiten an der anlage</t>
+          <t>leoni</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht</t>
+          <t>leoni störung</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht</t>
+          <t>leoni störung</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht (reparaturen seitens robtech)</t>
+          <t>leoni-fehler</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht (reparaturen seitens robtech)</t>
+          <t>leoni-fehler</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht / zuviel abrieb im fronius überm fass draht bleibt stecken, robotertechniker informiert</t>
+          <t>lichtbogen konnte nicht erzeugt werden</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht / zuviel abrieb im fronius überm fass draht bleibt stecken, robotertechniker informiert</t>
+          <t>lichtbogen konnte nicht erzeugt werden</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -1726,12 +1726,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht klöckner draht</t>
+          <t>mehrere stw 5 knoten op50 ist langsamer &amp; ( 5.ten knoten umsetzen)</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht klöckner draht</t>
+          <t>mehrere stw 5 knoten op50 ist langsamer &amp; ( 5.ten knoten umsetzen)</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -1741,57 +1741,57 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht, viel abrieb, strömdüse festgebrannt</t>
+          <t>mes - absturz keine etiketten-manuel ausdruken</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>probleme mit schweißdraht, viel abrieb, strömdüse festgebrannt</t>
+          <t>mes - absturz keine etiketten-manuel ausdruken</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>probleme mit stromdüse</t>
+          <t>mes - absturz keine etiketten=&gt; keine aufräge im puffer</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>probleme mit stromdüse</t>
+          <t>mes - absturz keine etiketten=&gt; keine aufräge im puffer</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>probleme mit stromdüse / gasdüse, erneuert</t>
+          <t>mitarbeitergespräch mit früh und spätschicht</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>probleme mit stromdüse / gasdüse, erneuert</t>
+          <t>mitarbeitergespräch mit früh und spätschicht</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>qs nacharbeitszelle + bauteil in anlage ausmessen</t>
+          <t>mittelnaht mangelhaft</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>qs nacharbeitszelle + bauteil in anlage ausmessen</t>
+          <t>mittelnaht mangelhaft</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -1801,42 +1801,42 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>qs-prüfplan</t>
+          <t>mittelnaht schlecht robotertechniker informiert</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>qs-prüfplan</t>
+          <t>mittelnaht schlecht robotertechniker informiert</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>quertraverse fährt nicht in position</t>
+          <t>not-aus</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>quertraverse fährt nicht in position</t>
+          <t>not-aus</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>r03 störung im programmablauf</t>
+          <t>not-aus folgefehler beseitigen</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>r03 störung im programmablauf</t>
+          <t>not-aus folgefehler beseitigen</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -1846,42 +1846,42 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>r05 , sensor im op130.1 und op30 wackelkontakt. robtech informiert</t>
+          <t>not-aus-durch monteur op100 folgefehler beseitigen</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>r05 , sensor im op130.1 und op30 wackelkontakt. robtech informiert</t>
+          <t>not-aus-durch monteur op100 folgefehler beseitigen</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>r05 fährt nach optimierungsarbeiten vom bmb kollision in op30 , ganzer greifer beschädigt und verbogen</t>
+          <t>nur 1 skid aktiv</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>r05 fährt nach optimierungsarbeiten vom bmb kollision in op30 , ganzer greifer beschädigt und verbogen</t>
+          <t>nur 1 skid aktiv</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>r05 greiferstörung</t>
+          <t>nur ein schweißer=&gt; ein schweißer für heckrungne ausgeliehen</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>r05 greiferstörung</t>
+          <t>nur ein schweißer=&gt; ein schweißer für heckrungne ausgeliehen</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -1891,27 +1891,27 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>r05 greiferstörung robotertechniker in der anlage</t>
+          <t>obenquerträger+trapezblech 5mm spalt=&gt; schweißnähte mangelhaft</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>r05 greiferstörung robotertechniker in der anlage</t>
+          <t>obenquerträger+trapezblech 5mm spalt=&gt; schweißnähte mangelhaft</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>r05 programmablauf störung/instandsetzung informiert</t>
+          <t>op10</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>r05 programmablauf störung/instandsetzung informiert</t>
+          <t>op10</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -1921,27 +1921,27 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>r05-programmablauf gestört</t>
+          <t>op10. r. kein vakuum-bleche manuell laden</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>r05-programmablauf gestört</t>
+          <t>op10. r. kein vakuum-bleche manuell laden</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>r06 l4 schweißstörungen</t>
+          <t>op120.1 auf passiv gestellt, reparaturarbeiten</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>r06 l4 schweißstörungen</t>
+          <t>op120.1 auf passiv gestellt, reparaturarbeiten</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -1951,102 +1951,102 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>r06(r07 collision detected</t>
+          <t>op130.2 auf passiv gestellt, reparaturarbeiten ( zylinder tauschen)</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>r06(r07 collision detected</t>
+          <t>op130.2 auf passiv gestellt, reparaturarbeiten ( zylinder tauschen)</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>r06/r07 kollisionen</t>
+          <t>optimierungsarbeiten an der anlage</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>r06/r07 kollisionen</t>
+          <t>optimierungsarbeiten an der anlage</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>r6/r7 kollision ,kabelbruch in der elektrik</t>
+          <t>probleme mit schweißdraht</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>r6/r7 kollision ,kabelbruch in der elektrik</t>
+          <t>probleme mit schweißdraht</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2</v>
+        <v>47</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>reparatur seitens robtech</t>
+          <t>probleme mit schweißdraht (reparaturen seitens robtech)</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>reparatur seitens robtech</t>
+          <t>probleme mit schweißdraht (reparaturen seitens robtech)</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>reparaturarbeiten-durch robtechs</t>
+          <t>probleme mit schweißdraht / zuviel abrieb im fronius überm fass draht bleibt stecken, robotertechniker informiert</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>reparaturarbeiten-durch robtechs</t>
+          <t>probleme mit schweißdraht / zuviel abrieb im fronius überm fass draht bleibt stecken, robotertechniker informiert</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>roboter fährt nicht los, robotertechniker informiert</t>
+          <t>probleme mit schweißdraht klöckner draht</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>roboter fährt nicht los, robotertechniker informiert</t>
+          <t>probleme mit schweißdraht klöckner draht</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>robotertechniker teacht schweißnähte nach</t>
+          <t>probleme mit schweißdraht, viel abrieb, strömdüse festgebrannt</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>robotertechniker teacht schweißnähte nach</t>
+          <t>probleme mit schweißdraht, viel abrieb, strömdüse festgebrannt</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -2056,42 +2056,42 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>rungen nachmontieren</t>
+          <t>probleme mit stromdüse</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>rungen nachmontieren</t>
+          <t>probleme mit stromdüse</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>rungen suchen</t>
+          <t>probleme mit stromdüse / gasdüse, erneuert</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>rungen suchen</t>
+          <t>probleme mit stromdüse / gasdüse, erneuert</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>schlitten abgesagt, spanner querträger oben defekt</t>
+          <t>qs nacharbeitszelle + bauteil in anlage ausmessen</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>schlitten abgesagt, spanner querträger oben defekt</t>
+          <t>qs nacharbeitszelle + bauteil in anlage ausmessen</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -2101,12 +2101,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>schlitten kollidiert mit trapezblechen</t>
+          <t>qs- führt vermessung der bauteile durch</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>schlitten kollidiert mit trapezblechen</t>
+          <t>qs- führt vermessung der bauteile durch</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -2116,27 +2116,27 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>schweißdraht wechseln</t>
+          <t>qs-prüfplan</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>schweißdraht wechseln</t>
+          <t>qs-prüfplan</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>schweißdrahtfass leer -gewechselt, drahtseele reinigen</t>
+          <t>quertraverse fährt nicht in position</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>schweißdrahtfass leer -gewechselt, drahtseele reinigen</t>
+          <t>quertraverse fährt nicht in position</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -2146,87 +2146,87 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>schweißstörung</t>
+          <t>r03 störung im programmablauf</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>schweißstörung</t>
+          <t>r03 störung im programmablauf</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>schweißstörung am fronius</t>
+          <t>r05 , sensor im op130.1 und op30 wackelkontakt. robtech informiert</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>schweißstörung am fronius</t>
+          <t>r05 , sensor im op130.1 und op30 wackelkontakt. robtech informiert</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>schweißstörung am fronius drahtfehler</t>
+          <t>r05 fährt nach optimierungsarbeiten vom bmb kollision in op30 , ganzer greifer beschädigt und verbogen</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>schweißstörung am fronius drahtfehler</t>
+          <t>r05 fährt nach optimierungsarbeiten vom bmb kollision in op30 , ganzer greifer beschädigt und verbogen</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>schweißstörung am fronius wegen draht</t>
+          <t>r05 greiferstörung</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>schweißstörung am fronius wegen draht</t>
+          <t>r05 greiferstörung</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>schweißstörung durch bauteil</t>
+          <t>r05 greiferstörung robotertechniker in der anlage</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>schweißstörung durch bauteil</t>
+          <t>r05 greiferstörung robotertechniker in der anlage</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>schweißt nicht mehr. robtech informiert</t>
+          <t>r05 programmablauf störung/instandsetzung informiert</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>schweißt nicht mehr. robtech informiert</t>
+          <t>r05 programmablauf störung/instandsetzung informiert</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -2236,12 +2236,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>sensoren ab- und anschrauben</t>
+          <t>r05-programmablauf gestört</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>sensoren ab- und anschrauben</t>
+          <t>r05-programmablauf gestört</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -2251,12 +2251,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>sensoren für stützen schalten nicht</t>
+          <t>r06 l4 schweißstörungen</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>sensoren für stützen schalten nicht</t>
+          <t>r06 l4 schweißstörungen</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -2266,42 +2266,42 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>sensoren schalten durchgehend</t>
+          <t>r06(r07 collision detected</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>sensoren schalten durchgehend</t>
+          <t>r06(r07 collision detected</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>skid passiv umbaumaßnahmen bmb; qs</t>
+          <t>r06/r07 kollisionen</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>skid passiv umbaumaßnahmen bmb; qs</t>
+          <t>r06/r07 kollisionen</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>softwareendschalter achse3</t>
+          <t>r6/r7 kollision ,kabelbruch in der elektrik</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>softwareendschalter achse3</t>
+          <t>r6/r7 kollision ,kabelbruch in der elektrik</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -2311,42 +2311,42 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>spanner nicht richtig geschlossen</t>
+          <t>reparatur greifer</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>spanner nicht richtig geschlossen</t>
+          <t>reparatur greifer</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>spanner oben, verriegelung</t>
+          <t>reparatur seitens robtech</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>spanner oben, verriegelung</t>
+          <t>reparatur seitens robtech</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>stirnwände 515102786 r06+r07 sollgeschwindigkeit a4 überschritten</t>
+          <t>reparatur seitens robtech/anlagenbereich reinigen/wochenplan</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>stirnwände 515102786 r06+r07 sollgeschwindigkeit a4 überschritten</t>
+          <t>reparatur seitens robtech/anlagenbereich reinigen/wochenplan</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -2356,12 +2356,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>stirnwände mit 5 knoten r03 kollisionen</t>
+          <t>reparaturarbeiten-durch robtechs</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>stirnwände mit 5 knoten r03 kollisionen</t>
+          <t>reparaturarbeiten-durch robtechs</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -2371,12 +2371,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>stirnwände nachmontieren</t>
+          <t>roboter fährt nicht los, robotertechniker informiert</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>stirnwände nachmontieren</t>
+          <t>roboter fährt nicht los, robotertechniker informiert</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -2386,12 +2386,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>streik</t>
+          <t>robotertechniker teacht schweißnähte nach</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>streik</t>
+          <t>robotertechniker teacht schweißnähte nach</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -2401,42 +2401,42 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>strom und gasdüse getauscht</t>
+          <t>rungen nachmontieren</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>strom und gasdüse getauscht</t>
+          <t>rungen nachmontieren</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>stw stützen andrücken störung ( vorrichtung nicht weit genug gefahren )</t>
+          <t>rungen suchen</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>stw stützen andrücken störung ( vorrichtung nicht weit genug gefahren )</t>
+          <t>rungen suchen</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>störung bei knoten schweißen</t>
+          <t>schlitten abgesagt, spanner querträger oben defekt</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>störung bei knoten schweißen</t>
+          <t>schlitten abgesagt, spanner querträger oben defekt</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -2446,147 +2446,147 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>störung beim abholen aus op120</t>
+          <t>schlitten kollidiert mit trapezblechen</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>störung beim abholen aus op120</t>
+          <t>schlitten kollidiert mit trapezblechen</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>störungen/anlage leer</t>
+          <t>schweißdraht wechseln</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>störungen/anlage leer</t>
+          <t>schweißdraht wechseln</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>stütze andrücken störung</t>
+          <t>schweißdrahtfass leer -gewechselt, drahtseele reinigen</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>stütze andrücken störung</t>
+          <t>schweißdrahtfass leer -gewechselt, drahtseele reinigen</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>stütze andrücken störung bei jeder l4 stirnwand</t>
+          <t>schweißstörung</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>stütze andrücken störung bei jeder l4 stirnwand</t>
+          <t>schweißstörung</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>stütze anschweißen nachteachen</t>
+          <t>schweißstörung am fronius</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>stütze anschweißen nachteachen</t>
+          <t>schweißstörung am fronius</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>suchfahrt</t>
+          <t>schweißstörung am fronius drahtfehler</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>suchfahrt</t>
+          <t>schweißstörung am fronius drahtfehler</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>tauschbox</t>
+          <t>schweißstörung am fronius wegen draht</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>tauschbox</t>
+          <t>schweißstörung am fronius wegen draht</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>teachen durch robotertechnker l4</t>
+          <t>schweißstörung durch bauteil</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>teachen durch robotertechnker l4</t>
+          <t>schweißstörung durch bauteil</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>teachen durch robotertechnker l5</t>
+          <t>schweißstörungen</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>teachen durch robotertechnker l5</t>
+          <t>schweißstörungen</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>trapezbleche beladen</t>
+          <t>schweißt nicht mehr. robtech informiert</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>trapezbleche beladen</t>
+          <t>schweißt nicht mehr. robtech informiert</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -2596,132 +2596,132 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern</t>
+          <t>sensoren ab- und anschrauben</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern</t>
+          <t>sensoren ab- und anschrauben</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern aufträge unterbrechen/freigeben</t>
+          <t>sensoren für stützen schalten nicht</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern aufträge unterbrechen/freigeben</t>
+          <t>sensoren für stützen schalten nicht</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern sensoren an-/abklemmen</t>
+          <t>sensoren schalten durchgehend</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern sensoren an-/abklemmen</t>
+          <t>sensoren schalten durchgehend</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern/sensoren an-/abklemmen</t>
+          <t>skid passiv umbaumaßnahmen bmb; qs</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern sensoren an-/abklemmen</t>
+          <t>skid passiv umbaumaßnahmen bmb; qs</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern-sensoren ab/anklemmen</t>
+          <t>softwareendschalter achse3</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern-sensoren ab/anklemmen</t>
+          <t>softwareendschalter achse3</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
+          <t>spanner nicht richtig geschlossen</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
+          <t>spanner nicht richtig geschlossen</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern-sensoren ab-/anklemmen</t>
+          <t>spanner oben, verriegelung</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
+          <t>spanner oben, verriegelung</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern sensoren ab-/anklemmen</t>
+          <t>stirnwände 515102786 r06+r07 sollgeschwindigkeit a4 überschritten</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
+          <t>stirnwände 515102786 r06+r07 sollgeschwindigkeit a4 überschritten</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>trapezbleche einlafern/sensoren ab-/anklemmen</t>
+          <t>stirnwände mit 5 knoten</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
+          <t>stirnwände mit 5 knoten</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -2731,57 +2731,57 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern=&gt; sensoren ab-/anklemmen</t>
+          <t>stirnwände mit 5 knoten r03 kollisionen</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>trapezbleche einlagern=&gt; sensoren ab-/anklemmen</t>
+          <t>stirnwände mit 5 knoten r03 kollisionen</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>trapezbleche laden-sensoren ab-/anklemmen</t>
+          <t>stirnwände mit eckrungen montieren</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>trapezbleche laden-sensoren ab-/anklemmen</t>
+          <t>stirnwände mit eckrungen montieren</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>trapezbleche nass/bleche manuell laden</t>
+          <t>stirnwände nachmontieren</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>trapezbleche nass/bleche manuell laden</t>
+          <t>stirnwände nachmontieren</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>trapezbleche nicht nah genug an questräger oben gefahren ohne störungsmeldung. robotertechniker informiert</t>
+          <t>streik</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>trapezbleche nicht nah genug an questräger oben gefahren ohne störungsmeldung. robotertechniker informiert</t>
+          <t>streik</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -2791,87 +2791,87 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>trapezbleche oben rechte seite nicht gespannt/angedrück</t>
+          <t>strom und gasdüse getauscht</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>trapezbleche oben rechte seite nicht gespannt/angedrück</t>
+          <t>strom und gasdüse getauscht</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>trapezbleche tauschen und sensoren abschrauben</t>
+          <t>stw stützen andrücken störung ( vorrichtung nicht weit genug gefahren )</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>trapezbleche tauschen und sensoren abschrauben</t>
+          <t>stw stützen andrücken störung ( vorrichtung nicht weit genug gefahren )</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden</t>
+          <t>störung bei knoten schweißen</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden</t>
+          <t>störung bei knoten schweißen</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>69</v>
+        <v>2</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden / material ölig</t>
+          <t>störung beim abholen aus op120</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden / material ölig</t>
+          <t>störung beim abholen aus op120</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden / vakuumkreis weiss</t>
+          <t>störungen-gestoppt durch r03</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden / vakuumkreis weiss</t>
+          <t>störungen-gestoppt durch r03</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden / wasser zwischen den blechen</t>
+          <t>störungen/anlage leer</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden / wasser zwischen den blechen</t>
+          <t>störungen/anlage leer</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -2881,27 +2881,27 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden in op 120-1</t>
+          <t>stütze andrücken störung</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden in op 120-1</t>
+          <t>stütze andrücken störung</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden, bleche kleben aneinander</t>
+          <t>stütze andrücken störung bei jeder l4 stirnwand</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden, bleche kleben aneinander</t>
+          <t>stütze andrücken störung bei jeder l4 stirnwand</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -2911,12 +2911,12 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden, bleche werden nicht richtig angesaug</t>
+          <t>stütze anschweißen nachteachen</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden, bleche werden nicht richtig angesaug</t>
+          <t>stütze anschweißen nachteachen</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -2926,255 +2926,780 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden, robotertechniker informiert</t>
+          <t>tauschbox</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>vakuum nicht vorhanden, robotertechniker informiert</t>
+          <t>tauschbox</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>vakuumkreis - vakuum nicht vorhanden</t>
+          <t>tauschbox/wartungsplan</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>vakuumkreis - vakuum nicht vorhanden</t>
+          <t>tauschbox/wartungsplan</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>vakuumkreis 1 schaltet nicht</t>
+          <t>teachen durch robotertechnker l4</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>vakuumkreis 1 schaltet nicht</t>
+          <t>teachen durch robotertechnker l4</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>vermessung skids op120/130 qs, bmb, robotertechnik in der anlage</t>
+          <t>teachen durch robotertechnker l5</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>vermessung skids op120/130 qs, bmb, robotertechnik in der anlage</t>
+          <t>teachen durch robotertechnker l5</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>warten auf eckrungen</t>
+          <t>trapezbleche 230(1028,5 mm breite) mittelnaht hällt nicht, bleche können nicht gespannt werden</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>warten auf eckrungen</t>
+          <t>trapezbleche 230(1028,5 mm breite) mittelnaht hällt nicht, bleche können nicht gespannt werden</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>warten auf eckrungen von der eckrungenanlage</t>
+          <t>trapezbleche beladen</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>warten auf eckrungen von der eckrungenanlage</t>
+          <t>trapezbleche beladen</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>warten auf eckrungen; reiniegung</t>
+          <t>trapezbleche einlagern</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>warten auf eckrungen; reiniegung</t>
+          <t>trapezbleche einlagern</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>warten auf rungen</t>
+          <t>trapezbleche einlagern aufträge unterbrechen/freigeben</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>warten auf rungen</t>
+          <t>trapezbleche einlagern aufträge unterbrechen/freigeben</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>warten auf trapezbleche</t>
+          <t>trapezbleche einlagern sensoren an-/abklemmen</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>warten auf trapezbleche</t>
+          <t>trapezbleche einlagern sensoren an-/abklemmen</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>wartungsplan</t>
+          <t>trapezbleche einlagern/sensoren an-/abklemmen</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>wartungsplan</t>
+          <t>trapezbleche einlagern sensoren an-/abklemmen</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>147</v>
+        <v>3</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>wartungsplan/tauschbox</t>
+          <t>trapezbleche einlagern-sensoren ab/anklemmen</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>wartungsplan/tauschbox</t>
+          <t>trapezbleche einlagern-sensoren ab/anklemmen</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>werkzeug einschließen und anlage ausschalten</t>
+          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>werkzeug einschließen und anlage ausschalten</t>
+          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>werkzeuge bereitstellen/wartungsplan/tauschbox</t>
+          <t>trapezbleche einlagern-sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>werkzeuge bereitstellen/wartungsplan/tauschbox</t>
+          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>werkzeuge verstauen/anlage ausschalten</t>
+          <t>trapezbleche einlagern sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>werkzeuge verstauen/anlage ausschalten</t>
+          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>wöchentliche reinigung</t>
+          <t>trapezbleche einlafern/sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>wöchentliche reinigung</t>
+          <t>trapezbleche einlagern/sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>zylinder für gravierer defekt/ instandsetzung informiert</t>
+          <t>trapezbleche einlagern=&gt; sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>zylinder für gravierer defekt/ instandsetzung informiert</t>
+          <t>trapezbleche einlagern=&gt; sensoren ab-/anklemmen</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
+          <t>trapezbleche laden-sensoren ab-/anklemmen</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>trapezbleche laden-sensoren ab-/anklemmen</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>trapezbleche nass/bleche manuell laden</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>trapezbleche nass/bleche manuell laden</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>trapezbleche nicht nah genug an questräg</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>trapezbleche nicht nah genug an questräg</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>trapezbleche nicht nah genug an questräger oben gefahren ohne störungsmeldung. robotertechniker informiert</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>trapezbleche nicht nah genug an questräger oben gefahren ohne störungsmeldung. robotertechniker informiert</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>trapezbleche oben rechte seite nicht gespannt/angedrück</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>trapezbleche oben rechte seite nicht gespannt/angedrück</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>trapezbleche tauschen und sensoren abschrauben</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>trapezbleche tauschen und sensoren abschrauben</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden ( bleche kleben aneinander )</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden ( bleche kleben aneinander )</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden ( belche kleben aneinander )</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden ( bleche kleben aneinander )</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden / material ölig</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden / material ölig</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden / vakuumkreis weiss</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden / vakuumkreis weiss</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden / wasser zwischen den blechen</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden / wasser zwischen den blechen</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden dreck auf dem trapezblech</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden dreck auf dem trapezblech</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden in op 120-1</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden in op 120-1</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden op 10 l bleche kleben aneinander</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden op 10 l bleche kleben aneinander</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden, bleche kleben aneinander</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden, bleche kleben aneinander</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden, bleche kleben zusammen( bleche sind nass )</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden, bleche kleben zusammen( bleche sind nass )</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden, bleche werden nicht richtig angesaug</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden, bleche werden nicht richtig angesaug</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden, robotertechniker informiert</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>vakuum nicht vorhanden, robotertechniker informiert</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>vakuumkreis - vakuum nicht vorhanden</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>vakuumkreis - vakuum nicht vorhanden</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>vakuumkreis 1 schaltet nicht</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>vakuumkreis 1 schaltet nicht</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>vermessung skids op120/130 qs, bmb, robotertechnik in der anlage</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>vermessung skids op120/130 qs, bmb, robotertechnik in der anlage</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>warten auf bereitschafts robotertechniker, reaparaturarbeiten</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>warten auf bereitschafts robotertechniker, reaparaturarbeiten</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>warten auf eckrungen</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>warten auf eckrungen</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>warten auf eckrungen von der eckrungenanlage</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>warten auf eckrungen von der eckrungenanlage</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>warten auf eckrungen; reiniegung</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>warten auf eckrungen; reiniegung</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>warten auf rungen</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>warten auf rungen</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>warten auf trapezbleche</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>warten auf trapezbleche</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>wartungsplan</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>wartungsplan</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>wartungsplan/tauschbox</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>wartungsplan/tauschbox</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>werkzeug einschließen und anlage ausschalten</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>werkzeug einschließen und anlage ausschalten</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>werkzeuge bereitstellen/wartungsplan/tauschbox</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>werkzeuge bereitstellen/wartungsplan/tauschbox</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>werkzeuge verstauen/anlage ausschalten</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>werkzeuge verstauen/anlage ausschalten</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>wöchentliche reinigung</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>wöchentliche reinigung</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>zylinder für gravierer defekt/ instandsetzung informiert</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>zylinder für gravierer defekt/ instandsetzung informiert</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
           <t>zündfehler</t>
         </is>
       </c>
-      <c r="B184" t="inlineStr">
+      <c r="B219" t="inlineStr">
         <is>
           <t>zündfehler</t>
         </is>
       </c>
-      <c r="C184" t="n">
+      <c r="C219" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>